<commit_message>
PNG to powerpoint added
</commit_message>
<xml_diff>
--- a/Hoe lang moet ik nog wachten/Hoe lang moet ik nog wachten.xlsx
+++ b/Hoe lang moet ik nog wachten/Hoe lang moet ik nog wachten.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\henkj\Documents\GitHub\RandomRepository\Hoe lang moet ik nog wachten\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72F56F0-FCA4-41B7-8CC4-4E5C57F3AAC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448FED51-5A03-4F9A-A557-32956344054E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="2" r:id="rId1"/>
@@ -391,58 +391,58 @@
                 <c:formatCode>dd\-mm\-yyyy" "hh":"mm</c:formatCode>
                 <c:ptCount val="986"/>
                 <c:pt idx="0">
-                  <c:v>46135.640972222223</c:v>
+                  <c:v>46131.893055555556</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>46135.642361111109</c:v>
+                  <c:v>46131.894444444442</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>46135.644444444442</c:v>
+                  <c:v>46131.895833333336</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>46135.649305555555</c:v>
+                  <c:v>46131.899305555555</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>46135.654166666667</c:v>
+                  <c:v>46131.900694444441</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>46135.65625</c:v>
+                  <c:v>46131.902777777781</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>46135.660416666666</c:v>
+                  <c:v>46131.904166666667</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>46135.663888888892</c:v>
+                  <c:v>46131.90625</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>46135.625</c:v>
+                  <c:v>46131.906944444447</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>46135.625</c:v>
+                  <c:v>46131.908333333333</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>46135.625</c:v>
+                  <c:v>46131.909722222219</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>46135.625</c:v>
+                  <c:v>46131.911111111112</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>46135.625</c:v>
+                  <c:v>46131.914583333331</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>46135.625</c:v>
+                  <c:v>46131.875</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>46135.625</c:v>
+                  <c:v>46131.875</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>46135.625</c:v>
+                  <c:v>46131.875</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>46135.625</c:v>
+                  <c:v>46131.875</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>46135.625</c:v>
+                  <c:v>46131.875</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -454,28 +454,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="986"/>
                 <c:pt idx="0">
-                  <c:v>154</c:v>
+                  <c:v>31591</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>157</c:v>
+                  <c:v>31646</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>161</c:v>
+                  <c:v>31691</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>172</c:v>
+                  <c:v>31839</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>183</c:v>
+                  <c:v>31901</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>187</c:v>
+                  <c:v>31990</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>196</c:v>
+                  <c:v>32045</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>204</c:v>
+                  <c:v>32112</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>32156</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>32223</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>32273</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>32384</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>32487</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1040,18 +1055,18 @@
       </c>
       <c r="K1">
         <f>SLOPE(G:G,F:F)</f>
-        <v>4.5828200921557553E-4</v>
+        <v>2.3609957188638396E-5</v>
       </c>
       <c r="M1" s="12">
         <f>3600*K1*24</f>
-        <v>39.595565596225725</v>
+        <v>2.0399003010983572</v>
       </c>
       <c r="N1" t="s">
         <v>5</v>
       </c>
       <c r="O1" s="11">
         <f>1/M1</f>
-        <v>2.5255353344297741E-2</v>
+        <v>0.4902200364701958</v>
       </c>
       <c r="P1" t="s">
         <v>18</v>
@@ -1065,43 +1080,43 @@
         <v>4</v>
       </c>
       <c r="C2" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D2" s="3">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E2" s="3">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F2" s="3">
-        <v>154</v>
+        <v>31591</v>
       </c>
       <c r="G2" s="4">
         <f t="shared" ref="G2:G3" si="0">DATE(A2,B2,C2)+TIME(D2,E2,0)</f>
-        <v>46135.640972222223</v>
+        <v>46131.893055555556</v>
       </c>
       <c r="H2" s="10">
         <f t="shared" ref="H2:H19" si="1">((G2-$K$2)/$K$1-F2)</f>
-        <v>-0.16923316454477799</v>
+        <v>-12.985694606326433</v>
       </c>
       <c r="J2" t="s">
         <v>1</v>
       </c>
       <c r="K2" s="1">
         <f>INTERCEPT(G:G,F:F)</f>
-        <v>46135.570474349319</v>
+        <v>46131.147499989704</v>
       </c>
       <c r="L2" s="1"/>
       <c r="M2" s="12">
         <f>M1/60</f>
-        <v>0.65992609327042873</v>
+        <v>3.3998338351639283E-2</v>
       </c>
       <c r="N2" t="s">
         <v>6</v>
       </c>
       <c r="O2" s="11">
         <f>1/M2</f>
-        <v>1.5153212006578647</v>
+        <v>29.413202188211748</v>
       </c>
       <c r="P2" t="s">
         <v>7</v>
@@ -1115,24 +1130,24 @@
         <v>4</v>
       </c>
       <c r="C3" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3" s="3">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E3" s="3">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F3" s="3">
-        <v>157</v>
+        <v>31646</v>
       </c>
       <c r="G3" s="4">
         <f t="shared" si="0"/>
-        <v>46135.642361111109</v>
+        <v>46131.894444444442</v>
       </c>
       <c r="H3" s="10">
         <f t="shared" si="1"/>
-        <v>-0.13859076922688018</v>
+        <v>-9.1592903463242692</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
@@ -1143,30 +1158,30 @@
         <v>4</v>
       </c>
       <c r="C4" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4" s="3">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E4" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F4" s="3">
-        <v>161</v>
+        <v>31691</v>
       </c>
       <c r="G4" s="4">
         <f t="shared" ref="G4:G12" si="2">DATE(A4,B4,C4)+TIME(D4,E4,0)</f>
-        <v>46135.644444444442</v>
+        <v>46131.895833333336</v>
       </c>
       <c r="H4" s="10">
         <f t="shared" si="1"/>
-        <v>0.40737283168826366</v>
+        <v>4.6671142218510795</v>
       </c>
       <c r="J4" t="s">
         <v>2</v>
       </c>
       <c r="K4" s="7">
-        <v>321</v>
+        <v>36131</v>
       </c>
       <c r="L4" s="7"/>
     </row>
@@ -1178,31 +1193,31 @@
         <v>4</v>
       </c>
       <c r="C5" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D5" s="3">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E5" s="3">
         <v>35</v>
       </c>
       <c r="F5" s="3">
-        <v>172</v>
+        <v>31839</v>
       </c>
       <c r="G5" s="4">
         <f t="shared" si="2"/>
-        <v>46135.649305555555</v>
+        <v>46131.899305555555</v>
       </c>
       <c r="H5" s="10">
         <f t="shared" si="1"/>
-        <v>1.4621239115825801E-2</v>
+        <v>3.7331250259449007</v>
       </c>
       <c r="J5" t="s">
         <v>3</v>
       </c>
       <c r="K5" s="1">
         <f>K2+K1*K4</f>
-        <v>46135.717582874277</v>
+        <v>46132.000551352889</v>
       </c>
       <c r="L5" s="1"/>
     </row>
@@ -1214,31 +1229,31 @@
         <v>4</v>
       </c>
       <c r="C6" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D6" s="3">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E6" s="3">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F6" s="3">
-        <v>183</v>
+        <v>31901</v>
       </c>
       <c r="G6" s="4">
         <f t="shared" si="2"/>
-        <v>46135.654166666667</v>
+        <v>46131.900694444441</v>
       </c>
       <c r="H6" s="10">
         <f t="shared" si="1"/>
-        <v>-0.37813035345661206</v>
+        <v>0.55952928594706464</v>
       </c>
       <c r="J6" t="s">
         <v>4</v>
       </c>
       <c r="K6" s="2">
         <f>CORREL(G:G,F:F)</f>
-        <v>0.99990159209756047</v>
+        <v>0.99851898442333265</v>
       </c>
       <c r="L6" s="2"/>
       <c r="O6" s="13"/>
@@ -1251,24 +1266,24 @@
         <v>4</v>
       </c>
       <c r="C7" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D7" s="3">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E7" s="3">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F7" s="3">
-        <v>187</v>
+        <v>31990</v>
       </c>
       <c r="G7" s="4">
         <f t="shared" si="2"/>
-        <v>46135.65625</v>
+        <v>46131.902777777781</v>
       </c>
       <c r="H7" s="10">
         <f t="shared" si="1"/>
-        <v>0.16783324745853179</v>
+        <v>-0.20086386179173132</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.35">
@@ -1279,24 +1294,24 @@
         <v>4</v>
       </c>
       <c r="C8" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D8" s="3">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E8" s="3">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="F8" s="3">
-        <v>196</v>
+        <v>32045</v>
       </c>
       <c r="G8" s="4">
         <f t="shared" si="2"/>
-        <v>46135.660416666666</v>
+        <v>46131.904166666667</v>
       </c>
       <c r="H8" s="10">
         <f t="shared" si="1"/>
-        <v>0.25976044928884789</v>
+        <v>3.6255403982104326</v>
       </c>
       <c r="J8" s="8" t="s">
         <v>15</v>
@@ -1310,24 +1325,24 @@
         <v>4</v>
       </c>
       <c r="C9" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D9" s="3">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E9" s="3">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="F9" s="3">
-        <v>204</v>
+        <v>32112</v>
       </c>
       <c r="G9" s="4">
         <f t="shared" si="2"/>
-        <v>46135.663888888892</v>
+        <v>46131.90625</v>
       </c>
       <c r="H9" s="10">
         <f t="shared" si="1"/>
-        <v>-0.16363353860148777</v>
+        <v>24.86514694230209</v>
       </c>
       <c r="J9" s="8" t="s">
         <v>16</v>
@@ -1341,18 +1356,24 @@
         <v>4</v>
       </c>
       <c r="C10" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D10" s="3">
-        <v>15</v>
+        <v>21</v>
+      </c>
+      <c r="E10" s="3">
+        <v>46</v>
+      </c>
+      <c r="F10" s="3">
+        <v>32156</v>
       </c>
       <c r="G10" s="4">
         <f t="shared" si="2"/>
-        <v>46135.625</v>
+        <v>46131.906944444447</v>
       </c>
       <c r="H10" s="10">
         <f t="shared" si="1"/>
-        <v>118.97837921785464</v>
+        <v>10.278349226391583</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.35">
@@ -1363,18 +1384,24 @@
         <v>4</v>
       </c>
       <c r="C11" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D11" s="3">
-        <v>15</v>
+        <v>21</v>
+      </c>
+      <c r="E11" s="3">
+        <v>48</v>
+      </c>
+      <c r="F11" s="3">
+        <v>32223</v>
       </c>
       <c r="G11" s="4">
         <f t="shared" si="2"/>
-        <v>46135.625</v>
+        <v>46131.908333333333</v>
       </c>
       <c r="H11" s="10">
         <f t="shared" si="1"/>
-        <v>118.97837921785464</v>
+        <v>2.1047534863937472</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
@@ -1385,18 +1412,24 @@
         <v>4</v>
       </c>
       <c r="C12" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D12" s="3">
-        <v>15</v>
+        <v>21</v>
+      </c>
+      <c r="E12" s="3">
+        <v>50</v>
+      </c>
+      <c r="F12" s="3">
+        <v>32273</v>
       </c>
       <c r="G12" s="4">
         <f t="shared" si="2"/>
-        <v>46135.625</v>
+        <v>46131.909722222219</v>
       </c>
       <c r="H12" s="10">
         <f t="shared" si="1"/>
-        <v>118.97837921785464</v>
+        <v>10.931157746395911</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.35">
@@ -1407,18 +1440,24 @@
         <v>4</v>
       </c>
       <c r="C13" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D13" s="3">
-        <v>15</v>
+        <v>21</v>
+      </c>
+      <c r="E13" s="3">
+        <v>52</v>
+      </c>
+      <c r="F13" s="3">
+        <v>32384</v>
       </c>
       <c r="G13" s="4">
         <f t="shared" ref="G13" si="3">DATE(A13,B13,C13)+TIME(D13,E13,0)</f>
-        <v>46135.625</v>
+        <v>46131.911111111112</v>
       </c>
       <c r="H13" s="10">
         <f t="shared" si="1"/>
-        <v>118.97837921785464</v>
+        <v>-41.24243768542874</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.35">
@@ -1429,18 +1468,24 @@
         <v>4</v>
       </c>
       <c r="C14" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D14" s="3">
-        <v>15</v>
+        <v>21</v>
+      </c>
+      <c r="E14" s="3">
+        <v>57</v>
+      </c>
+      <c r="F14" s="3">
+        <v>32487</v>
       </c>
       <c r="G14" s="4">
         <f t="shared" ref="G14:G16" si="4">DATE(A14,B14,C14)+TIME(D14,E14,0)</f>
-        <v>46135.625</v>
+        <v>46131.914583333331</v>
       </c>
       <c r="H14" s="10">
         <f t="shared" si="1"/>
-        <v>118.97837921785464</v>
+        <v>2.823573118665081</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
@@ -1451,18 +1496,18 @@
         <v>4</v>
       </c>
       <c r="C15" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D15" s="3">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G15" s="4">
         <f t="shared" si="4"/>
-        <v>46135.625</v>
+        <v>46131.875</v>
       </c>
       <c r="H15" s="10">
         <f t="shared" si="1"/>
-        <v>118.97837921785464</v>
+        <v>30813.271048472772</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.35">
@@ -1473,18 +1518,18 @@
         <v>4</v>
       </c>
       <c r="C16" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D16" s="3">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G16" s="4">
         <f t="shared" si="4"/>
-        <v>46135.625</v>
+        <v>46131.875</v>
       </c>
       <c r="H16" s="10">
         <f t="shared" si="1"/>
-        <v>118.97837921785464</v>
+        <v>30813.271048472772</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.35">
@@ -1495,18 +1540,18 @@
         <v>4</v>
       </c>
       <c r="C17" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D17" s="3">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G17" s="4">
         <f t="shared" ref="G17:G19" si="5">DATE(A17,B17,C17)+TIME(D17,E17,0)</f>
-        <v>46135.625</v>
+        <v>46131.875</v>
       </c>
       <c r="H17" s="10">
         <f t="shared" si="1"/>
-        <v>118.97837921785464</v>
+        <v>30813.271048472772</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
@@ -1517,18 +1562,18 @@
         <v>4</v>
       </c>
       <c r="C18" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D18" s="3">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G18" s="4">
         <f t="shared" si="5"/>
-        <v>46135.625</v>
+        <v>46131.875</v>
       </c>
       <c r="H18" s="10">
         <f t="shared" si="1"/>
-        <v>118.97837921785464</v>
+        <v>30813.271048472772</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
@@ -1539,18 +1584,18 @@
         <v>4</v>
       </c>
       <c r="C19" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D19" s="3">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G19" s="4">
         <f t="shared" si="5"/>
-        <v>46135.625</v>
+        <v>46131.875</v>
       </c>
       <c r="H19" s="10">
         <f t="shared" si="1"/>
-        <v>118.97837921785464</v>
+        <v>30813.271048472772</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">

</xml_diff>